<commit_message>
added recording for BBS Webinar: Optimizing Multiple Comparisons in Sequential and Non-Sequential Clinical Trials (Mar 9th, 2026)
</commit_message>
<xml_diff>
--- a/data/seminars.xlsx
+++ b/data/seminars.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schaej17\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D24ACD6-4629-410B-ABB8-B1FE5211163B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C68C5C-6688-4C5C-8492-2C3AF10BCCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1802" uniqueCount="1440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1803" uniqueCount="1441">
   <si>
     <t>Anja Schiel</t>
   </si>
@@ -4352,6 +4352,9 @@
   </si>
   <si>
     <t xml:space="preserve">American University, Washington DC, U.S.A. </t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=iu2amaqKMPc</t>
   </si>
 </sst>
 </file>
@@ -5122,7 +5125,9 @@
       <c r="B2" s="3" t="s">
         <v>1435</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="19" t="s">
+        <v>1440</v>
+      </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -25432,9 +25437,10 @@
     <hyperlink ref="L47" r:id="rId9" xr:uid="{6767DC4E-7DED-4CE9-B535-CB410788F1A2}"/>
     <hyperlink ref="C33" r:id="rId10" xr:uid="{962F91A3-71A2-4A72-9D8E-E9EF28200F39}"/>
     <hyperlink ref="L18" r:id="rId11" xr:uid="{9A2DD3EE-226E-4666-B380-3D214C636894}"/>
+    <hyperlink ref="C2" r:id="rId12" xr:uid="{6D3E4E88-1022-4D21-8782-789C865EE45E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
-  <drawing r:id="rId13"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>